<commit_message>
Updated template with coordinate systems. Last part of PDB-208.
git-svn-id: file:///repo/applications/FRED/branches/mikevdg_importer@45335 976ac4c7-77c1-46cc-9d05-16a3bd20634c
</commit_message>
<xml_diff>
--- a/fred-main-webapp/src/main/resources/fred_template.xlsx
+++ b/fred-main-webapp/src/main/resources/fred_template.xlsx
@@ -3,12 +3,13 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="19126"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="10_ncr:100000_{FD76FD8B-8952-48AF-93B3-78836DCB1DE3}" xr6:coauthVersionLast="31" xr6:coauthVersionMax="31" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="10_ncr:100000_{CCB5AECD-8D28-4EAA-9168-2230D7A41311}" xr6:coauthVersionLast="31" xr6:coauthVersionMax="31" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="_Cover_sheet" sheetId="1" r:id="rId1"/>
+    <sheet name="_Usage_Instructions" sheetId="1" r:id="rId1"/>
+    <sheet name="_Coordinate_Systems" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -20,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="108" uniqueCount="108">
   <si>
     <t>FRED Importer</t>
   </si>
@@ -100,26 +101,257 @@
     <t>Hacking the drop-down columns</t>
   </si>
   <si>
-    <t>Drop-down items have the format "Description / ID", where ID is a numeric database identifier. The ID is (usually) mandatory and should match an ID from the database. The importer (usually) ignores the Description. This may change in a later release of the importer.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">The lists can be edited, but only if the Importer and FRED know how to process the elements you put in there. </t>
-  </si>
-  <si>
-    <t>There is a hidden sheet called "_Lists". A sheet will be ignored if it's name starts with an underscore. Drop-down list cells have a constraint on them that only allows items to be selected from this list.</t>
-  </si>
-  <si>
     <t>The constraints are a standard Excel feature, visible in the "Data Validation" button in the "Data" toolbar.</t>
   </si>
   <si>
     <t>Columns each have a particular data validation constraint on them:</t>
+  </si>
+  <si>
+    <t>Coordinate Systems</t>
+  </si>
+  <si>
+    <t>The "Coordinate System" column only contains the most common coordinate systems. If you want to enter data using another coordinate system, copy and paste a value from the list below.</t>
+  </si>
+  <si>
+    <t>Amuri 2000 Local Circuit / 2</t>
+  </si>
+  <si>
+    <t>Amuri Local Circuit Metric / 1</t>
+  </si>
+  <si>
+    <t>Auckland Island TM / 67</t>
+  </si>
+  <si>
+    <t>Bay of Plenty 2000 Local Circuit / 47</t>
+  </si>
+  <si>
+    <t>Bay of Plenty Local Circuit Metric / 46</t>
+  </si>
+  <si>
+    <t>Bluff 2000 Local Circuit / 4</t>
+  </si>
+  <si>
+    <t>Bluff Local Circuit Metric / 3</t>
+  </si>
+  <si>
+    <t>Buller 2000 Local Circuit / 6</t>
+  </si>
+  <si>
+    <t>Buller Local circuit Metric / 5</t>
+  </si>
+  <si>
+    <t>Campbell Island TM / 68</t>
+  </si>
+  <si>
+    <t>Chatham Island Grid / 7</t>
+  </si>
+  <si>
+    <t>Collingwood 2000 Local Circuit / 9</t>
+  </si>
+  <si>
+    <t>Collingwood Local Circuit Metric / 8</t>
+  </si>
+  <si>
+    <t>Gawler 2000 Local Circuit / 13</t>
+  </si>
+  <si>
+    <t>Gawler Local Circuit Metric / 12</t>
+  </si>
+  <si>
+    <t>Grey 2000 Local Circuit / 15</t>
+  </si>
+  <si>
+    <t>Grey Local Circuit Metric / 14</t>
+  </si>
+  <si>
+    <t>Hawkes Bay 2000 Local Circuit / 19</t>
+  </si>
+  <si>
+    <t>Hawkes Bay Local Circuit Metric / 18</t>
+  </si>
+  <si>
+    <t>Hokitika 2000 Local Circuit / 21</t>
+  </si>
+  <si>
+    <t>Hokitika Local Circuit Metric / 20</t>
+  </si>
+  <si>
+    <t>Jacksons Bay 2000 Local Circuit / 23</t>
+  </si>
+  <si>
+    <t>Jacksons Bay Local Circuit Metric / 22</t>
+  </si>
+  <si>
+    <t>Karamea 2000 Local Circuit / 25</t>
+  </si>
+  <si>
+    <t>Karamea Local Circuit Metric / 24</t>
+  </si>
+  <si>
+    <t>Lat/Long Chatham Island Datum / 30</t>
+  </si>
+  <si>
+    <t>Lat/long GD2000 Datum / 28</t>
+  </si>
+  <si>
+    <t>Lat/long GD49 Datum / 29</t>
+  </si>
+  <si>
+    <t>Lat/long WGS84 Datum / 73</t>
+  </si>
+  <si>
+    <t>Lindis Peak 2000 Local Circuit / 27</t>
+  </si>
+  <si>
+    <t>Lindis Peak Local Circuit Metric / 26</t>
+  </si>
+  <si>
+    <t>Marlborough 2000 Local Circuit / 32</t>
+  </si>
+  <si>
+    <t>Marlborough Local Circuit Metric / 31</t>
+  </si>
+  <si>
+    <t>Mount Nicholas 2000 Local Circuit / 37</t>
+  </si>
+  <si>
+    <t>Mount Nicholas Local Circuit Metric / 36</t>
+  </si>
+  <si>
+    <t>Mount Pleasant 2000 Local Circuit / 45</t>
+  </si>
+  <si>
+    <t>Mount Pleasant Local Circuit Metric / 44</t>
+  </si>
+  <si>
+    <t>Mount York 2000 Local Circuit / 65</t>
+  </si>
+  <si>
+    <t>Mount York Local Circuit Metric / 64</t>
+  </si>
+  <si>
+    <t>Mt Eden 2000 Local Circuit / 11</t>
+  </si>
+  <si>
+    <t>Mt Eden Local Circuit Metric / 10</t>
+  </si>
+  <si>
+    <t>NZ Map Grid - Full / 38</t>
+  </si>
+  <si>
+    <t>NZ Map Grid - Trunc. / 16</t>
+  </si>
+  <si>
+    <t>NZ North Island Yard Grid / 70</t>
+  </si>
+  <si>
+    <t>NZ South Island Yard Grid / 33</t>
+  </si>
+  <si>
+    <t>NZ Transverse Mercator / 71</t>
+  </si>
+  <si>
+    <t>NZMS1 North Island Grid Ref / 69</t>
+  </si>
+  <si>
+    <t>NZMS1 South Island Grid Ref / 17</t>
+  </si>
+  <si>
+    <t>NZTopo50 / 72</t>
+  </si>
+  <si>
+    <t>Nelson 2000 Local Circuit / 35</t>
+  </si>
+  <si>
+    <t>Nelson Local Circuit Metric / 34</t>
+  </si>
+  <si>
+    <t>New Caledonia Transverse Mercator / 74</t>
+  </si>
+  <si>
+    <t>North Taieri 2000 Local Circuit / 51</t>
+  </si>
+  <si>
+    <t>North Taieri Local Circuit Metric / 50</t>
+  </si>
+  <si>
+    <t>Not A System / 76</t>
+  </si>
+  <si>
+    <t>Observation Point 2000 Local Circuit / 40</t>
+  </si>
+  <si>
+    <t>Observation Point Local Circuit Metric / 39</t>
+  </si>
+  <si>
+    <t>Okarito 2000 Local Circuit / 42</t>
+  </si>
+  <si>
+    <t>Okarito Local Circuit Metric / 41</t>
+  </si>
+  <si>
+    <t>Other - Specify details / 43</t>
+  </si>
+  <si>
+    <t>Poverty Bay 2000 Local Circuit / 49</t>
+  </si>
+  <si>
+    <t>Poverty Bay Local Circuit Metric / 48</t>
+  </si>
+  <si>
+    <t>Remote Site / 66</t>
+  </si>
+  <si>
+    <t>Taranaki 2000 Local Circuit / 53</t>
+  </si>
+  <si>
+    <t>Taranaki Local Circuit Metric / 52</t>
+  </si>
+  <si>
+    <t>Timaru 2000 Local Circuit / 55</t>
+  </si>
+  <si>
+    <t>Timaru Local Circuit Metric / 54</t>
+  </si>
+  <si>
+    <t>Tuhirangi 2000 Local Circuit / 57</t>
+  </si>
+  <si>
+    <t>Tuhirangi Local Circuit Metric / 56</t>
+  </si>
+  <si>
+    <t>Wairarapa 2000 Local Circuit / 59</t>
+  </si>
+  <si>
+    <t>Wairarapa Local Circuit Metric / 58</t>
+  </si>
+  <si>
+    <t>Wanganui 2000 Local Circuit / 61</t>
+  </si>
+  <si>
+    <t>Wanganui Local Circuit Metric / 60</t>
+  </si>
+  <si>
+    <t>Wellington 2000 Local Circuit / 63</t>
+  </si>
+  <si>
+    <t>Wellington Local Circuit Metric / 62</t>
+  </si>
+  <si>
+    <t>There is a hidden sheet called "_Lists". A sheet will be ignored by the importer if it's name starts with an underscore. Drop-down list cells have a constraint on them that only allows items to be selected from this list.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The lists can be edited by, for example, you, but only if the Importer and FRED know how to process the elements you put in there. </t>
+  </si>
+  <si>
+    <t>Drop-down items have the format "Description / ID", where ID is a numeric database identifier. The ID is (usually) mandatory and should match an ID from the database. The importer (usually) ignores the description. This may change in a later release of the importer.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -156,6 +388,14 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="3">
     <fill>
@@ -183,7 +423,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -201,6 +441,10 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -493,7 +737,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:1" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:1" ht="11.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A2" s="1"/>
     </row>
     <row r="3" spans="1:1" ht="30" x14ac:dyDescent="0.25">
@@ -512,7 +756,7 @@
     <row r="6" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A6" s="3"/>
     </row>
-    <row r="7" spans="1:1" ht="30" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:1" ht="46.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="s">
         <v>3</v>
       </c>
@@ -522,7 +766,7 @@
     </row>
     <row r="9" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A9" s="3" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
     </row>
     <row r="10" spans="1:1" x14ac:dyDescent="0.25">
@@ -563,7 +807,7 @@
     </row>
     <row r="18" spans="1:1" ht="30" x14ac:dyDescent="0.25">
       <c r="A18" s="3" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
     </row>
     <row r="19" spans="1:1" x14ac:dyDescent="0.25">
@@ -614,7 +858,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="35" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:1" ht="30" x14ac:dyDescent="0.25">
       <c r="A35" s="6" t="s">
         <v>19</v>
       </c>
@@ -649,19 +893,420 @@
         <v>25</v>
       </c>
     </row>
-    <row r="45" spans="1:1" ht="30" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:1" ht="45" x14ac:dyDescent="0.25">
       <c r="A45" s="6" t="s">
-        <v>28</v>
+        <v>105</v>
       </c>
     </row>
     <row r="47" spans="1:1" ht="30" x14ac:dyDescent="0.25">
       <c r="A47" s="6" t="s">
-        <v>27</v>
+        <v>106</v>
       </c>
     </row>
     <row r="49" spans="1:1" ht="45" x14ac:dyDescent="0.25">
       <c r="A49" s="6" t="s">
-        <v>26</v>
+        <v>107</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B9AA6572-7E82-403D-BC74-CA95650F531C}">
+  <dimension ref="A1:C78"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="75.85546875" customWidth="1"/>
+    <col min="3" max="3" width="23" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" ht="25.5" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A1" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="C1" s="8"/>
+    </row>
+    <row r="2" spans="1:3" ht="55.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="7" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="17" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="18" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="19" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="20" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="21" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="22" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="23" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="24" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="25" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="26" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="27" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="28" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="29" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="30" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="31" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="32" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="33" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="34" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="35" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="36" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A36" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="37" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A37" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="38" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A38" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="39" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A39" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="40" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A40" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="41" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A41" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="42" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A42" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="43" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A43" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="44" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A44" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="45" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A45" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="46" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A46" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="47" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A47" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="48" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A48" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="49" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A49" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="50" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A50" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="51" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A51" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="52" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A52" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="53" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A53" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="54" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A54" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="55" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A55" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="56" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A56" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="57" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A57" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="58" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A58" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="59" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A59" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="60" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A60" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="61" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A61" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="62" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A62" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="63" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A63" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="64" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A64" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="65" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A65" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="66" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A66" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="67" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A67" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="68" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A68" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="69" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A69" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="70" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A70" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="71" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A71" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="72" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A72" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="73" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A73" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="74" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A74" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="75" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A75" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="76" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A76" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="77" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A77" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="78" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A78" t="s">
+        <v>104</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
PDB-212: updating the cover sheet with feedback from Chris.
git-svn-id: file:///repo/applications/FRED/branches/mikevdg_importer@45449 976ac4c7-77c1-46cc-9d05-16a3bd20634c
</commit_message>
<xml_diff>
--- a/fred-main-webapp/src/main/resources/fred_template.xlsx
+++ b/fred-main-webapp/src/main/resources/fred_template.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="19126"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="10_ncr:100000_{CCB5AECD-8D28-4EAA-9168-2230D7A41311}" xr6:coauthVersionLast="31" xr6:coauthVersionMax="31" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="10_ncr:100000_{73048187-9CC3-47E2-9C8F-18EA9BDA9A5C}" xr6:coauthVersionLast="31" xr6:coauthVersionMax="31" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -32,9 +32,6 @@
     <t>Enter data into this spreadsheet. Each column heading has more information available about it if you hover the mouse pointer over it.</t>
   </si>
   <si>
-    <t xml:space="preserve">Do not rename the headings or add new headings. The importer relies on their exact names to process the spreadsheet. You may re-order headings, and if you know a column is optional then it can be removed. </t>
-  </si>
-  <si>
     <t>If you cut and paste entries, this might remove the constraints - try to always only "Paste Values". You can also edit or remove the constraints if you need to.</t>
   </si>
   <si>
@@ -53,9 +50,6 @@
     <t>• Some date columns are "Timestamps", meaning they allow dates and times.</t>
   </si>
   <si>
-    <t>• Drop-down columns allow only the entries given in the list. Some drop-down columns allow you to enter new values.</t>
-  </si>
-  <si>
     <t>Multi-Value Columns</t>
   </si>
   <si>
@@ -98,9 +92,6 @@
     <t>• Errors are shown in the logs with their row. The row number is in the leftmost column and the cell with the error is highlighted in orange.</t>
   </si>
   <si>
-    <t>Hacking the drop-down columns</t>
-  </si>
-  <si>
     <t>The constraints are a standard Excel feature, visible in the "Data Validation" button in the "Data" toolbar.</t>
   </si>
   <si>
@@ -338,13 +329,22 @@
     <t>Wellington Local Circuit Metric / 62</t>
   </si>
   <si>
-    <t>There is a hidden sheet called "_Lists". A sheet will be ignored by the importer if it's name starts with an underscore. Drop-down list cells have a constraint on them that only allows items to be selected from this list.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">The lists can be edited by, for example, you, but only if the Importer and FRED know how to process the elements you put in there. </t>
-  </si>
-  <si>
-    <t>Drop-down items have the format "Description / ID", where ID is a numeric database identifier. The ID is (usually) mandatory and should match an ID from the database. The importer (usually) ignores the description. This may change in a later release of the importer.</t>
+    <t>Do not rename the headings or add new headings. The importer relies on their exact names to process the spreadsheet. You can also adjust column widths and "hide" columns, although care should be taken so as not to overlook mandatory columns.</t>
+  </si>
+  <si>
+    <t>• Drop-down columns give you a list of options to choose from. Some drop-down columns only allow entries from the list. Other drop-down columns allow you to type in new entries.</t>
+  </si>
+  <si>
+    <t>Managing Drop-down Columns</t>
+  </si>
+  <si>
+    <t>Any sheet with a name that starts with an underscore ("_") will be ignored by the importer.</t>
+  </si>
+  <si>
+    <t>Drop-down list items have the format "Description / ID", where ID is a numeric database identifier. The ID is (usually) mandatory and should match an ID from the database. The importer (usually) ignores the description. This may change in a later release of the importer.</t>
+  </si>
+  <si>
+    <t>There is a hidden sheet called "_Lists". Do not modify this sheet; it is used for creating drop-down lists.</t>
   </si>
 </sst>
 </file>
@@ -423,7 +423,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -445,6 +445,9 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -756,9 +759,9 @@
     <row r="6" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A6" s="3"/>
     </row>
-    <row r="7" spans="1:1" ht="46.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="3" t="s">
-        <v>3</v>
+    <row r="7" spans="1:1" ht="45" x14ac:dyDescent="0.25">
+      <c r="A7" s="9" t="s">
+        <v>102</v>
       </c>
     </row>
     <row r="8" spans="1:1" x14ac:dyDescent="0.25">
@@ -766,7 +769,7 @@
     </row>
     <row r="9" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A9" s="3" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
     </row>
     <row r="10" spans="1:1" x14ac:dyDescent="0.25">
@@ -774,32 +777,32 @@
     </row>
     <row r="11" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A11" s="3" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="12" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A12" s="3" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="13" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A13" s="3" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="14" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A14" s="3" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="15" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A15" s="3" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="16" spans="1:1" ht="30" x14ac:dyDescent="0.25">
       <c r="A16" s="3" t="s">
-        <v>10</v>
+        <v>103</v>
       </c>
     </row>
     <row r="17" spans="1:1" x14ac:dyDescent="0.25">
@@ -807,7 +810,7 @@
     </row>
     <row r="18" spans="1:1" ht="30" x14ac:dyDescent="0.25">
       <c r="A18" s="3" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
     </row>
     <row r="19" spans="1:1" x14ac:dyDescent="0.25">
@@ -815,97 +818,97 @@
     </row>
     <row r="20" spans="1:1" ht="30" x14ac:dyDescent="0.25">
       <c r="A20" s="3" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="22" spans="1:1" ht="23.25" x14ac:dyDescent="0.35">
       <c r="A22" s="5" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
     </row>
     <row r="24" spans="1:1" ht="30" x14ac:dyDescent="0.25">
       <c r="A24" s="6" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
     </row>
     <row r="26" spans="1:1" ht="45" x14ac:dyDescent="0.25">
       <c r="A26" s="6" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
     </row>
     <row r="28" spans="1:1" ht="30" x14ac:dyDescent="0.25">
       <c r="A28" s="6" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
     </row>
     <row r="30" spans="1:1" ht="23.25" x14ac:dyDescent="0.35">
       <c r="A30" s="5" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
     </row>
     <row r="32" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A32" s="6" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
     </row>
     <row r="33" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A33" s="6" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
     </row>
     <row r="34" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A34" s="6" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
     </row>
     <row r="35" spans="1:1" ht="30" x14ac:dyDescent="0.25">
       <c r="A35" s="6" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
     </row>
     <row r="36" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A36" s="6" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
     </row>
     <row r="37" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A37" s="6" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
     </row>
     <row r="39" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A39" s="6" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
     </row>
     <row r="40" spans="1:1" ht="30" x14ac:dyDescent="0.25">
       <c r="A40" s="6" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
     </row>
     <row r="41" spans="1:1" ht="30" x14ac:dyDescent="0.25">
       <c r="A41" s="6" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
     </row>
     <row r="43" spans="1:1" ht="23.25" x14ac:dyDescent="0.35">
       <c r="A43" s="5" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="45" spans="1:1" ht="45" x14ac:dyDescent="0.25">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="45" spans="1:1" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A45" s="6" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="47" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A47" s="6" t="s">
         <v>105</v>
-      </c>
-    </row>
-    <row r="47" spans="1:1" ht="30" x14ac:dyDescent="0.25">
-      <c r="A47" s="6" t="s">
-        <v>106</v>
       </c>
     </row>
     <row r="49" spans="1:1" ht="45" x14ac:dyDescent="0.25">
       <c r="A49" s="6" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
     </row>
   </sheetData>
@@ -925,388 +928,388 @@
   <sheetData>
     <row r="1" spans="1:3" ht="25.5" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A1" s="1" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="C1" s="8"/>
     </row>
     <row r="2" spans="1:3" ht="55.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="7" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
     </row>
     <row r="17" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
     </row>
     <row r="18" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
     </row>
     <row r="19" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
     </row>
     <row r="20" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
     </row>
     <row r="21" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
     </row>
     <row r="22" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
     </row>
     <row r="23" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
     </row>
     <row r="24" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
     </row>
     <row r="25" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
     </row>
     <row r="26" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
     </row>
     <row r="27" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
     </row>
     <row r="28" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
     </row>
     <row r="29" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
     </row>
     <row r="30" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
     </row>
     <row r="31" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
     </row>
     <row r="32" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
     </row>
     <row r="33" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
     </row>
     <row r="34" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
     </row>
     <row r="35" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
     </row>
     <row r="36" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
     </row>
     <row r="37" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
     </row>
     <row r="38" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
     </row>
     <row r="39" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
     </row>
     <row r="40" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
     </row>
     <row r="41" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
     </row>
     <row r="42" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
     </row>
     <row r="43" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
     </row>
     <row r="44" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
     </row>
     <row r="45" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
     </row>
     <row r="46" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
     </row>
     <row r="47" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
     </row>
     <row r="48" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
     </row>
     <row r="49" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
     </row>
     <row r="50" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
     </row>
     <row r="51" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
     </row>
     <row r="52" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
     </row>
     <row r="53" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
     </row>
     <row r="54" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
     </row>
     <row r="55" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
     </row>
     <row r="56" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
     </row>
     <row r="57" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
     </row>
     <row r="58" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
     </row>
     <row r="59" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
-        <v>85</v>
+        <v>82</v>
       </c>
     </row>
     <row r="60" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
     </row>
     <row r="61" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
     </row>
     <row r="62" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
     </row>
     <row r="63" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
     </row>
     <row r="64" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
     </row>
     <row r="65" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
     </row>
     <row r="66" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
     </row>
     <row r="67" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
     </row>
     <row r="68" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
-        <v>94</v>
+        <v>91</v>
       </c>
     </row>
     <row r="69" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
     </row>
     <row r="70" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
     </row>
     <row r="71" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
     </row>
     <row r="72" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
-        <v>98</v>
+        <v>95</v>
       </c>
     </row>
     <row r="73" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
     </row>
     <row r="74" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
     </row>
     <row r="75" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
     </row>
     <row r="76" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
-        <v>102</v>
+        <v>99</v>
       </c>
     </row>
     <row r="77" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
-        <v>103</v>
+        <v>100</v>
       </c>
     </row>
     <row r="78" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
-        <v>104</v>
+        <v>101</v>
       </c>
     </row>
   </sheetData>

</xml_diff>